<commit_message>
Regen ODM v1 to v2 mapping config file (with yaml_to_xlsx_mapper.py)
</commit_message>
<xml_diff>
--- a/odm_map_maker/data/mapping_config_files/odm_v1_to_v2_mapping.xlsx
+++ b/odm_map_maker/data/mapping_config_files/odm_v1_to_v2_mapping.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="contacts" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="instruments" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="measures" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="organizations" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="polygons" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="protocols" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="qualityReports" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="samples" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="sites" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="wide_protocolSteps" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="enums" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="contacts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="instruments" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="measures" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="organizations" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="polygons" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="protocols" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="qualityReports" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="samples" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sites" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="wide_protocolSteps" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="enums" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>